<commit_message>
Implement ISO, UPPER_CASE and male/female
</commit_message>
<xml_diff>
--- a/injury_data.xlsx
+++ b/injury_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,237 +436,520 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>SEX</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Team</t>
+          <t>NAME</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Injury Date</t>
+          <t>CODE</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Return Date</t>
+          <t>INJURY_DATE</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Injury Location</t>
+          <t>RETURN_DATE</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Injury Side</t>
+          <t>INJURY_LOCATION</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Injury Type</t>
+          <t>INJURY_SIDE</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Occurrence</t>
+          <t>INJURY_TYPE</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Overuse/Trauma</t>
+          <t>OCCURRENCE</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Onset</t>
+          <t>OVERUSE_TRAUMA</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>ONSET</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>CONTACT</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Action Description</t>
+          <t>ACTION</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Re-injury</t>
+          <t>ACTION_DESCRIPTION</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Referee Sanction</t>
+          <t>RE_INJURY</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Diagnostic Examination</t>
+          <t>REFEREE_SANCTION</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Diagnosis</t>
+          <t>DIAGNOSTIC_EXAMINATION</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Surgery</t>
+          <t>DIAGNOSIS</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Menstrual Phase</t>
+          <t>SURGERY</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Oral Contraceptives</t>
+          <t>MENSTRUAL_PHASE</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Hormonal Contraceptives</t>
+          <t>ORAL_CONTRACEPTIVES</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Other Comments</t>
+          <t>HORMONAL_CONTRACEPTIVES</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>OTHER_COMMENTS</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>1.docx</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2.docx</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Luca F</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FC B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>xx11x</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2025-06-23</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Wrong date format</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Lower leg (incl. Achilles tendon)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Bilateral/central</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Muscle rupture/tear/strain**</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>N/A (gradual onset injury)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Overuse (repetitive mechanism)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Gradual onset</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>No foul, Opponent foul, Own foul, Yellow card, Red card</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Ultrasonography</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Should appear</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3.docx</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>All filled</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FC ALL</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>XXXXX</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2025-06-10</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-10-12</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Head, Abdomen, Elbow, Hip, Lower leg (incl. Achilles tendon), Neck, Lumbosacral, Forearm, Groin, Ankle, Chest, Shoulder, Wrist, Thigh, Foot, Thoracic spine, Upper arm, Hand, Knee</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Right, Left, Bilateral/central</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Concussion, Meniscus lesion, Haematoma/contusion/bruise (incl. compartment syndrome), Fracture (specify if stress fracture), Cartilage lesion, Nerve injury (central or peripheral other than concussion), Other bone injury (e.g., bone stress), Muscle rupture/tear/strain**, Dental injury*, Joint dislocation/subluxation*, Tendon rupture/tendinopathy, Vessel injury (excl. skin haematoma), Joint sprain (i.e., ligament/capsule), Abrasion, Bursitis, Arthritis/synovitis/capsulitis, Laceration, Overuse unspecified, Additional Injury</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Training, Match (min. of injury: 70), N/A (gradual onset injury), Football training, Football &amp; other training, League match, Friendly match, Other training, Reserve/youth team training, Champions League, Reserve/youth team match, National team, Other cup match</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Running/sprinting, Heading, Controlling the ball, Tackling other player, Blocked*, Twisting/turning, Landing (incl. jumping), Hit by ball, Tackled by other player, Use of arm/elbow*, Shooting/passing, Falling (incl. diving), Collision, Sliding/stretching*, Other player action</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Did everything</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>No foul, Opponent foul, Own foul, Yellow card, Red card</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Clinical only, X-ray, Ultrasonography, MRI, Other</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>DIagnosis</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Too many answers</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>xxxx_yy.docx</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>NAME SURNAME</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>TEAM_NAME</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>TEAM:CODE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2022-5-3</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2022-6-3</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2022-05-03</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2022-06-03</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Thigh</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Left</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Joint sprain (i.e., ligament/capsule)</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Match (min. of injury: 70), National team</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Trauma (acute mechanism)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Sudden onset</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Yes, direct contact (to injured body part)</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>Falling (incl. diving)</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>direct contact to the A-C joint on an unprotected fall</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>Opponent foul</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>MRI</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>A-C joint II degree sprain</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>